<commit_message>
Done with initial analysis
</commit_message>
<xml_diff>
--- a/Varied Parameters.xlsx
+++ b/Varied Parameters.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saividyud/Documents/GitHub/NASA_25-26_Rocket_Simulations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2383CFD6-DCC6-3643-B124-C276BF4C4981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61373FED-A075-A945-88BE-486AB1F1B2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="620" windowWidth="30240" windowHeight="17480" activeTab="1" xr2:uid="{D72F03AF-D0CB-7048-A263-60968BD6DCA1}"/>
+    <workbookView xWindow="-38400" yWindow="1400" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{D72F03AF-D0CB-7048-A263-60968BD6DCA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Options" sheetId="2" r:id="rId1"/>
     <sheet name="Parameter List" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="72">
   <si>
     <t>Parameter Name</t>
   </si>
@@ -180,15 +180,9 @@
     <t>Constant</t>
   </si>
   <si>
-    <t>[286, 302] K</t>
-  </si>
-  <si>
     <t>[0, 360) deg</t>
   </si>
   <si>
-    <t>Function Name</t>
-  </si>
-  <si>
     <t>[5, 10] deg</t>
   </si>
   <si>
@@ -198,65 +192,74 @@
     <t>28.5 in</t>
   </si>
   <si>
-    <t>6.125 in</t>
-  </si>
-  <si>
-    <t>{0, 45, 90} deg</t>
-  </si>
-  <si>
     <t>{0, 5, 10, 15, 20} mph</t>
   </si>
   <si>
-    <t>Nose Cone Shape Parameter</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>26 in</t>
-  </si>
-  <si>
-    <t>{Trapezoidal, Elliptical, Parallelogram, Swept Trapezoidal}</t>
-  </si>
-  <si>
-    <t>34 in</t>
-  </si>
-  <si>
-    <t>42 in</t>
-  </si>
-  <si>
     <t>0.1 in</t>
   </si>
   <si>
     <t>0.01 in</t>
   </si>
   <si>
-    <t>2.2 lbs</t>
-  </si>
-  <si>
-    <t>0.01 lbs</t>
-  </si>
-  <si>
-    <t>2.7 lbs</t>
-  </si>
-  <si>
-    <t>1.9 lbs</t>
-  </si>
-  <si>
-    <t>3.4 lbs</t>
-  </si>
-  <si>
     <t>500 Pa</t>
   </si>
   <si>
     <t>101325 Pa</t>
+  </si>
+  <si>
+    <t>{Swept, Tapered Swept, Trapezoidal, Elliptical}</t>
+  </si>
+  <si>
+    <t>2.52 lbs</t>
+  </si>
+  <si>
+    <t>33 in</t>
+  </si>
+  <si>
+    <t>31.5 in</t>
+  </si>
+  <si>
+    <t>2.41 lbs</t>
+  </si>
+  <si>
+    <t>3.32 lbs</t>
+  </si>
+  <si>
+    <t>43.5 in</t>
+  </si>
+  <si>
+    <t>6.12 in</t>
+  </si>
+  <si>
+    <t>2.03 lbs</t>
+  </si>
+  <si>
+    <t>[283, 302] K</t>
+  </si>
+  <si>
+    <t>Fin Thickness</t>
+  </si>
+  <si>
+    <t>0.25 in</t>
+  </si>
+  <si>
+    <t>Fin Mass</t>
+  </si>
+  <si>
+    <t>0.87 lbs</t>
+  </si>
+  <si>
+    <t>90 deg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -264,37 +267,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF9C5700"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -306,19 +285,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Bad" xfId="1" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -347,18 +320,17 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D43AC392-C9D8-814D-AE4E-23CC2E89DE4B}" name="Table2" displayName="Table2" ref="A1:F40" totalsRowShown="0">
-  <autoFilter ref="A1:F40" xr:uid="{D43AC392-C9D8-814D-AE4E-23CC2E89DE4B}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F20">
-    <sortCondition ref="C1:C40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D43AC392-C9D8-814D-AE4E-23CC2E89DE4B}" name="Table2" displayName="Table2" ref="A1:E21" totalsRowShown="0">
+  <autoFilter ref="A1:E21" xr:uid="{D43AC392-C9D8-814D-AE4E-23CC2E89DE4B}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F21">
+    <sortCondition ref="C1:C41"/>
   </sortState>
-  <tableColumns count="6">
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{3757E623-6D22-4D4A-BBD1-A15C4E60A30B}" name="Parameter Name"/>
     <tableColumn id="6" xr3:uid="{0FD49CFA-4811-0842-8E6C-1A597C08D0BB}" name="Parameter Type"/>
     <tableColumn id="3" xr3:uid="{3C16EC4D-5669-7A4D-AD96-E46CCBF91267}" name="Distribution Type"/>
     <tableColumn id="4" xr3:uid="{86896CA6-0B86-B647-9193-BA193206D17C}" name="Average Value"/>
     <tableColumn id="5" xr3:uid="{AC8CFD54-2B20-6B47-A5B6-F936482A8CAB}" name="Uncertainty"/>
-    <tableColumn id="2" xr3:uid="{CD05F7FD-1B28-9C47-BBCD-4621E4308051}" name="Function Name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -818,7 +790,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3BCF3C8-1C6B-A245-A02F-5C0ECA1A4145}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.33203125" customWidth="1"/>
@@ -846,9 +818,6 @@
       <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
-        <v>49</v>
-      </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -861,7 +830,7 @@
         <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -875,43 +844,46 @@
         <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
         <v>44</v>
       </c>
       <c r="D5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" t="s">
-        <v>69</v>
+        <v>65</v>
+      </c>
+      <c r="E5">
+        <v>0.05</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
         <v>42</v>
@@ -919,16 +891,16 @@
       <c r="C6" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>65</v>
+      <c r="D6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6">
+        <v>0.05</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
         <v>42</v>
@@ -936,16 +908,16 @@
       <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.01</v>
+      <c r="D7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7">
+        <v>0.05</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
@@ -954,18 +926,15 @@
         <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E8" t="s">
         <v>62</v>
       </c>
-      <c r="G8" t="s">
-        <v>57</v>
+      <c r="E8">
+        <v>0.05</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
         <v>42</v>
@@ -973,16 +942,16 @@
       <c r="C9" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>65</v>
+      <c r="D9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9">
+        <v>0.05</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>42</v>
@@ -990,16 +959,16 @@
       <c r="C10" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>65</v>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>42</v>
@@ -1007,16 +976,16 @@
       <c r="C11" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>65</v>
+      <c r="D11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>42</v>
@@ -1024,16 +993,16 @@
       <c r="C12" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>62</v>
+      <c r="D12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
         <v>42</v>
@@ -1041,16 +1010,19 @@
       <c r="C13" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>62</v>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>42</v>
@@ -1058,16 +1030,16 @@
       <c r="C14" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>62</v>
+      <c r="D14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>42</v>
@@ -1075,16 +1047,16 @@
       <c r="C15" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>63</v>
+      <c r="D15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
         <v>42</v>
@@ -1092,16 +1064,16 @@
       <c r="C16" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>63</v>
+      <c r="D16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s">
         <v>42</v>
@@ -1109,11 +1081,11 @@
       <c r="C17" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>63</v>
+      <c r="D17" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1127,7 +1099,7 @@
         <v>45</v>
       </c>
       <c r="D18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1141,21 +1113,35 @@
         <v>45</v>
       </c>
       <c r="D19" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="B20" t="s">
         <v>43</v>
       </c>
       <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" t="s">
         <v>45</v>
       </c>
-      <c r="D20" t="s">
-        <v>50</v>
+      <c r="D21" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1171,7 +1157,7 @@
           <x14:formula1>
             <xm:f>Options!$B$2:$B$4</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B40</xm:sqref>
+          <xm:sqref>B2:B21</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Done with all CDR analysis
</commit_message>
<xml_diff>
--- a/Varied Parameters.xlsx
+++ b/Varied Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saividyud/Documents/GitHub/NASA_25-26_Rocket_Simulations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61373FED-A075-A945-88BE-486AB1F1B2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613E7CED-DDCE-ED4B-B603-A893924F0DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1400" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{D72F03AF-D0CB-7048-A263-60968BD6DCA1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{D72F03AF-D0CB-7048-A263-60968BD6DCA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Options" sheetId="2" r:id="rId1"/>
@@ -252,7 +252,7 @@
     <t>0.87 lbs</t>
   </si>
   <si>
-    <t>90 deg</t>
+    <t>180 deg</t>
   </si>
 </sst>
 </file>

</xml_diff>